<commit_message>
feat(scheduler): English Net teacher weekly assignment for DAE102
- Add 'Net Teachers' sheet to Planning for Timetable.xlsx (Barrett + Chris Hon)
- DB schema: teachers.is_net flag; _load_net_teachers() reads the sheet
- New constants: _ENG_SUBJECT_CODE, _ENG_NET_MIN_BLOCKS=2, _ENG_MAX_TRAVEL_MIN=30,
  _ENG_TERMS, _ENG_WEEK_BLOCKS, _ENG_NET_EXEMPT_GROUPS={CS1,CS2,CS3,CS7}
- assign_english_weekly(): assigns teachers to 6 week-block slots per DAE102 class
  (2 terms x 3 blocks); prioritises Net teachers until min blocks met; enforces
  30-min travel cap for English teachers; CS1-3/CS7 exempt from Net requirement
- write_output_fast(): adds 'English Weekly' sheet with 10-column layout
- run_v4_from_bytes(): calls assign_english_weekly, adds Net shortfall warnings
- MASTER_PLAN.md: mark B3/B4/B5 fixed, add B6/J8/J9, update progression to V6.2
- change-log: document all 5 changes made today

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/Planning for Timetable.xlsx
+++ b/data/input/Planning for Timetable.xlsx
@@ -16,9 +16,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teacher load table with subject" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centre Room Allocation" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teacher Availability" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Net Teachers" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <externalReferences>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Class list answer'!$A$1:$L$109</definedName>
@@ -7363,6 +7364,41 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Teacher Name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Mr. Peter Barrett</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Mr. Chris Hon</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>